<commit_message>
Update MLB weather 2026-07-17 03:35 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v4_1_2026_07_18.xlsx
+++ b/mlb_weather_professional_v4_1_2026_07_18.xlsx
@@ -581,13 +581,13 @@
     <t>Density 73 | Wind 48 | Temp 62 | Altitude 64 | Confidence 73%</t>
   </si>
   <si>
-    <t>Density 73 | Wind 43 | Temp 55 | Altitude 63 | Confidence 89%</t>
+    <t>Density 73 | Wind 43 | Temp 55 | Altitude 63 | Confidence 87%</t>
   </si>
   <si>
     <t>Density 100 | Wind 41 | Temp 72 | Altitude 100 | Confidence 93%</t>
   </si>
   <si>
-    <t>Density 76 | Wind 74 | Temp 66 | Altitude 65 | Confidence 71%</t>
+    <t>Density 76 | Wind 74 | Temp 66 | Altitude 65 | Confidence 70%</t>
   </si>
   <si>
     <t>Density 61 | Wind 50 | Temp 74 | Altitude 56 | Confidence 90%</t>
@@ -599,7 +599,7 @@
     <t>Density 61 | Wind 50 | Temp 73 | Altitude 57 | Confidence 88%</t>
   </si>
   <si>
-    <t>Density 67 | Wind 77 | Temp 53 | Altitude 59 | Confidence 75%</t>
+    <t>Density 67 | Wind 77 | Temp 53 | Altitude 59 | Confidence 76%</t>
   </si>
   <si>
     <t>Density 84 | Wind 65 | Temp 68 | Altitude 72 | Confidence 85%</t>
@@ -614,7 +614,7 @@
     <t>Density 60 | Wind 45 | Temp 49 | Altitude 55 | Confidence 91%</t>
   </si>
   <si>
-    <t>Density 70 | Wind 65 | Temp 55 | Altitude 61 | Confidence 84%</t>
+    <t>Density 70 | Wind 65 | Temp 55 | Altitude 61 | Confidence 85%</t>
   </si>
   <si>
     <t>Density 67 | Wind 70 | Temp 60 | Altitude 61 | Confidence 90%</t>
@@ -635,18 +635,18 @@
     <t>IMPROVING RAPIDLY</t>
   </si>
   <si>
+    <t>WORSENING</t>
+  </si>
+  <si>
+    <t>IMPROVING</t>
+  </si>
+  <si>
+    <t>STEADY</t>
+  </si>
+  <si>
     <t>WORSENING RAPIDLY</t>
   </si>
   <si>
-    <t>STEADY</t>
-  </si>
-  <si>
-    <t>IMPROVING</t>
-  </si>
-  <si>
-    <t>WORSENING</t>
-  </si>
-  <si>
     <t>MODERATE</t>
   </si>
   <si>
@@ -665,49 +665,49 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-07-17 02:54:50 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:54:52 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:54:56 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:54:58 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:00 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:01 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:03 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:05 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:06 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:07 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:09 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:11 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:12 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:13 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-07-17 02:55:14 PM PDT</t>
+    <t>2026-07-17 03:35:06 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:07 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:12 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:14 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:15 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:16 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:18 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:19 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:20 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:21 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:22 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:23 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:24 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:25 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-07-17 03:35:26 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -1055,49 +1055,49 @@
     <t>10:07 PM PDT</t>
   </si>
   <si>
-    <t>2026-07-17 21:54:50 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:54:52 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:54:56 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:54:58 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:00 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:01 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:03 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:05 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:06 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:07 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:09 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:11 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:12 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:13 UTC</t>
-  </si>
-  <si>
-    <t>2026-07-17 21:55:14 UTC</t>
+    <t>2026-07-17 22:35:06 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:07 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:12 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:14 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:15 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:16 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:18 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:19 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:20 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:21 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:22 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:23 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:24 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:25 UTC</t>
+  </si>
+  <si>
+    <t>2026-07-17 22:35:26 UTC</t>
   </si>
   <si>
     <t>2026-07-17T20:02:20+00:00</t>
@@ -1974,7 +1974,7 @@
         <v>3.6</v>
       </c>
       <c r="AC2">
-        <v>75</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="AD2" t="s">
         <v>200</v>
@@ -2019,7 +2019,7 @@
         <v>203</v>
       </c>
       <c r="AR2">
-        <v>6.3</v>
+        <v>7.2</v>
       </c>
       <c r="AS2">
         <v>0</v>
@@ -2031,19 +2031,19 @@
         <v>208</v>
       </c>
       <c r="AV2">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
       <c r="AW2" t="s">
         <v>210</v>
       </c>
       <c r="AX2">
-        <v>17.1</v>
+        <v>17</v>
       </c>
       <c r="AY2" t="s">
         <v>214</v>
       </c>
       <c r="AZ2">
-        <v>112.5</v>
+        <v>152.8</v>
       </c>
       <c r="BA2">
         <v>5</v>
@@ -2111,7 +2111,7 @@
         <v>180</v>
       </c>
       <c r="V3">
-        <v>43.2</v>
+        <v>44</v>
       </c>
       <c r="W3">
         <v>56.6</v>
@@ -2174,10 +2174,10 @@
         <v>69.7</v>
       </c>
       <c r="AQ3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="AR3">
-        <v>4.2</v>
+        <v>-2.2</v>
       </c>
       <c r="AS3">
         <v>0</v>
@@ -2189,7 +2189,7 @@
         <v>209</v>
       </c>
       <c r="AV3">
-        <v>61.2</v>
+        <v>61.7</v>
       </c>
       <c r="AW3" t="s">
         <v>213</v>
@@ -2201,7 +2201,7 @@
         <v>215</v>
       </c>
       <c r="AZ3">
-        <v>63.6</v>
+        <v>103.8</v>
       </c>
       <c r="BA3">
         <v>5</v>
@@ -2269,7 +2269,7 @@
         <v>180</v>
       </c>
       <c r="V4">
-        <v>23.4</v>
+        <v>26.7</v>
       </c>
       <c r="W4">
         <v>53.1</v>
@@ -2290,7 +2290,7 @@
         <v>0.9</v>
       </c>
       <c r="AC4">
-        <v>88.8</v>
+        <v>87.2</v>
       </c>
       <c r="AD4" t="s">
         <v>201</v>
@@ -2335,7 +2335,7 @@
         <v>204</v>
       </c>
       <c r="AR4">
-        <v>-4</v>
+        <v>-3.4</v>
       </c>
       <c r="AS4">
         <v>0</v>
@@ -2347,13 +2347,13 @@
         <v>208</v>
       </c>
       <c r="AV4">
-        <v>31</v>
+        <v>32.8</v>
       </c>
       <c r="AW4" t="s">
         <v>210</v>
       </c>
       <c r="AX4">
-        <v>2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AY4" t="s">
         <v>216</v>
@@ -2493,7 +2493,7 @@
         <v>205</v>
       </c>
       <c r="AR5">
-        <v>1.3</v>
+        <v>2.6</v>
       </c>
       <c r="AS5">
         <v>0</v>
@@ -2511,13 +2511,13 @@
         <v>210</v>
       </c>
       <c r="AX5">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="AY5" t="s">
         <v>217</v>
       </c>
       <c r="AZ5">
-        <v>188.5</v>
+        <v>228.8</v>
       </c>
       <c r="BA5">
         <v>5</v>
@@ -2585,7 +2585,7 @@
         <v>180</v>
       </c>
       <c r="V6">
-        <v>61.3</v>
+        <v>59.8</v>
       </c>
       <c r="W6">
         <v>67.40000000000001</v>
@@ -2606,7 +2606,7 @@
         <v>5.2</v>
       </c>
       <c r="AC6">
-        <v>70.7</v>
+        <v>70.5</v>
       </c>
       <c r="AD6" t="s">
         <v>200</v>
@@ -2651,7 +2651,7 @@
         <v>203</v>
       </c>
       <c r="AR6">
-        <v>8.4</v>
+        <v>7.1</v>
       </c>
       <c r="AS6">
         <v>0</v>
@@ -2669,13 +2669,13 @@
         <v>213</v>
       </c>
       <c r="AX6">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
       <c r="AY6" t="s">
         <v>218</v>
       </c>
       <c r="AZ6">
-        <v>106.7</v>
+        <v>147</v>
       </c>
       <c r="BA6">
         <v>5</v>
@@ -2806,7 +2806,7 @@
         <v>47.2</v>
       </c>
       <c r="AQ7" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AR7">
         <v>3.3</v>
@@ -2827,13 +2827,13 @@
         <v>210</v>
       </c>
       <c r="AX7">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AY7" t="s">
         <v>219</v>
       </c>
       <c r="AZ7">
-        <v>213.2</v>
+        <v>253.5</v>
       </c>
       <c r="BA7">
         <v>5</v>
@@ -2991,7 +2991,7 @@
         <v>220</v>
       </c>
       <c r="AZ8">
-        <v>27.6</v>
+        <v>67.8</v>
       </c>
       <c r="BA8">
         <v>5</v>
@@ -3080,7 +3080,7 @@
         <v>0</v>
       </c>
       <c r="AC9">
-        <v>88.3</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="AD9" t="s">
         <v>201</v>
@@ -3122,7 +3122,7 @@
         <v>43.1</v>
       </c>
       <c r="AQ9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AR9">
         <v>3.3</v>
@@ -3149,7 +3149,7 @@
         <v>221</v>
       </c>
       <c r="AZ9">
-        <v>202</v>
+        <v>242.2</v>
       </c>
       <c r="BA9">
         <v>5</v>
@@ -3217,10 +3217,10 @@
         <v>180</v>
       </c>
       <c r="V10">
-        <v>55.5</v>
+        <v>58.1</v>
       </c>
       <c r="W10">
-        <v>65.2</v>
+        <v>65.3</v>
       </c>
       <c r="X10" t="s">
         <v>181</v>
@@ -3238,7 +3238,7 @@
         <v>4.6</v>
       </c>
       <c r="AC10">
-        <v>75.09999999999999</v>
+        <v>75.7</v>
       </c>
       <c r="AD10" t="s">
         <v>200</v>
@@ -3283,7 +3283,7 @@
         <v>203</v>
       </c>
       <c r="AR10">
-        <v>9.6</v>
+        <v>10.8</v>
       </c>
       <c r="AS10">
         <v>0</v>
@@ -3295,19 +3295,19 @@
         <v>209</v>
       </c>
       <c r="AV10">
-        <v>52.2</v>
+        <v>54.7</v>
       </c>
       <c r="AW10" t="s">
         <v>213</v>
       </c>
       <c r="AX10">
-        <v>30.1</v>
+        <v>30</v>
       </c>
       <c r="AY10" t="s">
         <v>222</v>
       </c>
       <c r="AZ10">
-        <v>164.2</v>
+        <v>204.4</v>
       </c>
       <c r="BA10">
         <v>5</v>
@@ -3396,7 +3396,7 @@
         <v>5.2</v>
       </c>
       <c r="AC11">
-        <v>85.2</v>
+        <v>85.3</v>
       </c>
       <c r="AD11" t="s">
         <v>200</v>
@@ -3438,10 +3438,10 @@
         <v>58.6</v>
       </c>
       <c r="AQ11" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="AR11">
-        <v>3.6</v>
+        <v>4.6</v>
       </c>
       <c r="AS11">
         <v>0</v>
@@ -3465,7 +3465,7 @@
         <v>223</v>
       </c>
       <c r="AZ11">
-        <v>208.7</v>
+        <v>248.9</v>
       </c>
       <c r="BA11">
         <v>5</v>
@@ -3533,7 +3533,7 @@
         <v>180</v>
       </c>
       <c r="V12">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="W12">
         <v>58.4</v>
@@ -3596,10 +3596,10 @@
         <v>57.5</v>
       </c>
       <c r="AQ12" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="AR12">
-        <v>7.4</v>
+        <v>-1</v>
       </c>
       <c r="AS12">
         <v>0</v>
@@ -3611,19 +3611,19 @@
         <v>210</v>
       </c>
       <c r="AV12">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="AW12" t="s">
         <v>210</v>
       </c>
       <c r="AX12">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
       <c r="AY12" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="AZ12">
-        <v>132.3</v>
+        <v>172.5</v>
       </c>
       <c r="BA12">
         <v>5</v>
@@ -3712,7 +3712,7 @@
         <v>1.3</v>
       </c>
       <c r="AC13">
-        <v>81.3</v>
+        <v>80.8</v>
       </c>
       <c r="AD13" t="s">
         <v>201</v>
@@ -3754,10 +3754,10 @@
         <v>78.40000000000001</v>
       </c>
       <c r="AQ13" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="AR13">
-        <v>-7.6</v>
+        <v>-4.8</v>
       </c>
       <c r="AS13">
         <v>0</v>
@@ -3775,13 +3775,13 @@
         <v>213</v>
       </c>
       <c r="AX13">
-        <v>27</v>
+        <v>26.9</v>
       </c>
       <c r="AY13" t="s">
         <v>224</v>
       </c>
       <c r="AZ13">
-        <v>112.8</v>
+        <v>153</v>
       </c>
       <c r="BA13">
         <v>5</v>
@@ -3912,10 +3912,10 @@
         <v>56.8</v>
       </c>
       <c r="AQ14" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="AR14">
-        <v>-2.2</v>
+        <v>-2.7</v>
       </c>
       <c r="AS14">
         <v>0</v>
@@ -3933,13 +3933,13 @@
         <v>210</v>
       </c>
       <c r="AX14">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="AY14" t="s">
         <v>225</v>
       </c>
       <c r="AZ14">
-        <v>208.3</v>
+        <v>248.5</v>
       </c>
       <c r="BA14">
         <v>5</v>
@@ -4007,7 +4007,7 @@
         <v>180</v>
       </c>
       <c r="V15">
-        <v>61.2</v>
+        <v>65.7</v>
       </c>
       <c r="W15">
         <v>62.3</v>
@@ -4028,7 +4028,7 @@
         <v>3.7</v>
       </c>
       <c r="AC15">
-        <v>84.2</v>
+        <v>84.7</v>
       </c>
       <c r="AD15" t="s">
         <v>200</v>
@@ -4073,7 +4073,7 @@
         <v>203</v>
       </c>
       <c r="AR15">
-        <v>6.7</v>
+        <v>6.2</v>
       </c>
       <c r="AS15">
         <v>0</v>
@@ -4085,7 +4085,7 @@
         <v>209</v>
       </c>
       <c r="AV15">
-        <v>55.5</v>
+        <v>58</v>
       </c>
       <c r="AW15" t="s">
         <v>213</v>
@@ -4097,7 +4097,7 @@
         <v>226</v>
       </c>
       <c r="AZ15">
-        <v>160.8</v>
+        <v>201</v>
       </c>
       <c r="BA15">
         <v>5</v>
@@ -4186,7 +4186,7 @@
         <v>4.5</v>
       </c>
       <c r="AC16">
-        <v>89.7</v>
+        <v>89.8</v>
       </c>
       <c r="AD16" t="s">
         <v>200</v>
@@ -4231,7 +4231,7 @@
         <v>203</v>
       </c>
       <c r="AR16">
-        <v>9.199999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="AS16">
         <v>0</v>
@@ -4255,7 +4255,7 @@
         <v>227</v>
       </c>
       <c r="AZ16">
-        <v>54.1</v>
+        <v>94.3</v>
       </c>
       <c r="BA16">
         <v>5</v>
@@ -4386,10 +4386,10 @@
         <v>73</v>
       </c>
       <c r="AQ17" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="AR17">
-        <v>3.4</v>
+        <v>3.8</v>
       </c>
       <c r="AS17">
         <v>0</v>
@@ -4407,13 +4407,13 @@
         <v>210</v>
       </c>
       <c r="AX17">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
       <c r="AY17" t="s">
         <v>228</v>
       </c>
       <c r="AZ17">
-        <v>6.4</v>
+        <v>46.6</v>
       </c>
       <c r="BA17">
         <v>5</v>
@@ -4805,10 +4805,10 @@
         <v>359</v>
       </c>
       <c r="J2">
-        <v>112.5</v>
+        <v>152.8</v>
       </c>
       <c r="K2">
-        <v>19.3</v>
+        <v>18.6</v>
       </c>
       <c r="L2">
         <v>5</v>
@@ -4850,7 +4850,7 @@
         <v>34.5</v>
       </c>
       <c r="Y2">
-        <v>77.59999999999999</v>
+        <v>77.7</v>
       </c>
       <c r="Z2">
         <v>64.40000000000001</v>
@@ -5056,10 +5056,10 @@
         <v>359</v>
       </c>
       <c r="J3">
-        <v>112.5</v>
+        <v>152.8</v>
       </c>
       <c r="K3">
-        <v>20.3</v>
+        <v>19.6</v>
       </c>
       <c r="L3">
         <v>5</v>
@@ -5071,7 +5071,7 @@
         <v>2.33</v>
       </c>
       <c r="O3">
-        <v>21.84</v>
+        <v>21.69</v>
       </c>
       <c r="P3">
         <v>3.2</v>
@@ -5143,7 +5143,7 @@
         <v>52.6</v>
       </c>
       <c r="AM3">
-        <v>32.1</v>
+        <v>32.2</v>
       </c>
       <c r="AN3">
         <v>0.008999999999999999</v>
@@ -5260,7 +5260,7 @@
         <v>208</v>
       </c>
       <c r="BZ3">
-        <v>17.1</v>
+        <v>17</v>
       </c>
       <c r="CA3" t="s">
         <v>210</v>
@@ -5307,10 +5307,10 @@
         <v>359</v>
       </c>
       <c r="J4">
-        <v>112.5</v>
+        <v>152.8</v>
       </c>
       <c r="K4">
-        <v>21.3</v>
+        <v>20.6</v>
       </c>
       <c r="L4">
         <v>5</v>
@@ -5322,7 +5322,7 @@
         <v>3.13</v>
       </c>
       <c r="O4">
-        <v>22.45</v>
+        <v>21.33</v>
       </c>
       <c r="P4">
         <v>5.4</v>
@@ -5349,10 +5349,10 @@
         <v>0.1667</v>
       </c>
       <c r="X4">
-        <v>43.8</v>
+        <v>43.4</v>
       </c>
       <c r="Y4">
-        <v>71.8</v>
+        <v>72</v>
       </c>
       <c r="Z4">
         <v>63.7</v>
@@ -5394,7 +5394,7 @@
         <v>84.90000000000001</v>
       </c>
       <c r="AM4">
-        <v>37.7</v>
+        <v>38.4</v>
       </c>
       <c r="AN4">
         <v>0.011</v>
@@ -5505,13 +5505,13 @@
         <v>40.2</v>
       </c>
       <c r="BX4">
-        <v>37.7</v>
+        <v>38.1</v>
       </c>
       <c r="BY4" t="s">
         <v>208</v>
       </c>
       <c r="BZ4">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
       <c r="CA4" t="s">
         <v>210</v>
@@ -5558,10 +5558,10 @@
         <v>359</v>
       </c>
       <c r="J5">
-        <v>112.5</v>
+        <v>152.8</v>
       </c>
       <c r="K5">
-        <v>22.3</v>
+        <v>21.6</v>
       </c>
       <c r="L5">
         <v>5</v>
@@ -5573,7 +5573,7 @@
         <v>2.71</v>
       </c>
       <c r="O5">
-        <v>24.35</v>
+        <v>22.6</v>
       </c>
       <c r="P5">
         <v>11.1</v>
@@ -5600,13 +5600,13 @@
         <v>0.1667</v>
       </c>
       <c r="X5">
-        <v>42.8</v>
+        <v>42.2</v>
       </c>
       <c r="Y5">
-        <v>72.5</v>
+        <v>72.8</v>
       </c>
       <c r="Z5">
-        <v>60.7</v>
+        <v>60.8</v>
       </c>
       <c r="AA5">
         <v>0.92</v>
@@ -5645,7 +5645,7 @@
         <v>89.09999999999999</v>
       </c>
       <c r="AM5">
-        <v>43</v>
+        <v>44.1</v>
       </c>
       <c r="AN5">
         <v>0.017</v>
@@ -5756,7 +5756,7 @@
         <v>41.8</v>
       </c>
       <c r="BX5">
-        <v>43.8</v>
+        <v>44.4</v>
       </c>
       <c r="BY5" t="s">
         <v>208</v>
@@ -5809,10 +5809,10 @@
         <v>360</v>
       </c>
       <c r="J6">
-        <v>63.6</v>
+        <v>103.8</v>
       </c>
       <c r="K6">
-        <v>20.4</v>
+        <v>19.7</v>
       </c>
       <c r="L6">
         <v>5</v>
@@ -5824,7 +5824,7 @@
         <v>4.35</v>
       </c>
       <c r="O6">
-        <v>32.17</v>
+        <v>30.84</v>
       </c>
       <c r="P6">
         <v>29.2</v>
@@ -5851,10 +5851,10 @@
         <v>0.3333</v>
       </c>
       <c r="X6">
-        <v>34.1</v>
+        <v>33.7</v>
       </c>
       <c r="Y6">
-        <v>71.7</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="Z6">
         <v>64.8</v>
@@ -5896,7 +5896,7 @@
         <v>62.2</v>
       </c>
       <c r="AM6">
-        <v>43.2</v>
+        <v>44</v>
       </c>
       <c r="AN6">
         <v>0.06</v>
@@ -6007,13 +6007,13 @@
         <v>39.5</v>
       </c>
       <c r="BX6">
-        <v>61.2</v>
+        <v>61.7</v>
       </c>
       <c r="BY6" t="s">
         <v>209</v>
       </c>
       <c r="BZ6">
-        <v>23.6</v>
+        <v>23.5</v>
       </c>
       <c r="CA6" t="s">
         <v>213</v>
@@ -6060,10 +6060,10 @@
         <v>360</v>
       </c>
       <c r="J7">
-        <v>63.6</v>
+        <v>103.8</v>
       </c>
       <c r="K7">
-        <v>21.4</v>
+        <v>20.7</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -6075,7 +6075,7 @@
         <v>4.56</v>
       </c>
       <c r="O7">
-        <v>28.1</v>
+        <v>29.03</v>
       </c>
       <c r="P7">
         <v>41.5</v>
@@ -6102,10 +6102,10 @@
         <v>0.3333</v>
       </c>
       <c r="X7">
-        <v>32.1</v>
+        <v>32.4</v>
       </c>
       <c r="Y7">
-        <v>72.8</v>
+        <v>72.7</v>
       </c>
       <c r="Z7">
         <v>57.7</v>
@@ -6147,7 +6147,7 @@
         <v>81.8</v>
       </c>
       <c r="AM7">
-        <v>57.8</v>
+        <v>57.2</v>
       </c>
       <c r="AN7">
         <v>0.035</v>
@@ -6243,7 +6243,7 @@
         <v>1.025</v>
       </c>
       <c r="BS7">
-        <v>66.7</v>
+        <v>66.8</v>
       </c>
       <c r="BT7">
         <v>54.1</v>
@@ -6258,7 +6258,7 @@
         <v>42.5</v>
       </c>
       <c r="BX7">
-        <v>60.3</v>
+        <v>60</v>
       </c>
       <c r="BY7" t="s">
         <v>209</v>
@@ -6311,10 +6311,10 @@
         <v>360</v>
       </c>
       <c r="J8">
-        <v>63.6</v>
+        <v>103.8</v>
       </c>
       <c r="K8">
-        <v>22.4</v>
+        <v>21.7</v>
       </c>
       <c r="L8">
         <v>5</v>
@@ -6326,7 +6326,7 @@
         <v>3.06</v>
       </c>
       <c r="O8">
-        <v>29.94</v>
+        <v>29.62</v>
       </c>
       <c r="P8">
         <v>42.1</v>
@@ -6353,7 +6353,7 @@
         <v>0.3333</v>
       </c>
       <c r="X8">
-        <v>25.5</v>
+        <v>25.3</v>
       </c>
       <c r="Y8">
         <v>74.7</v>
@@ -6398,7 +6398,7 @@
         <v>43.1</v>
       </c>
       <c r="AM8">
-        <v>55.2</v>
+        <v>55.6</v>
       </c>
       <c r="AN8">
         <v>0.008</v>
@@ -6509,7 +6509,7 @@
         <v>48.1</v>
       </c>
       <c r="BX8">
-        <v>45.5</v>
+        <v>45.7</v>
       </c>
       <c r="BY8" t="s">
         <v>209</v>
@@ -6562,10 +6562,10 @@
         <v>360</v>
       </c>
       <c r="J9">
-        <v>63.6</v>
+        <v>103.8</v>
       </c>
       <c r="K9">
-        <v>23.4</v>
+        <v>22.7</v>
       </c>
       <c r="L9">
         <v>5</v>
@@ -6577,7 +6577,7 @@
         <v>2.99</v>
       </c>
       <c r="O9">
-        <v>31.55</v>
+        <v>32.66</v>
       </c>
       <c r="P9">
         <v>5.4</v>
@@ -6604,13 +6604,13 @@
         <v>0.3333</v>
       </c>
       <c r="X9">
-        <v>25.1</v>
+        <v>25.5</v>
       </c>
       <c r="Y9">
-        <v>79.5</v>
+        <v>79.3</v>
       </c>
       <c r="Z9">
-        <v>27</v>
+        <v>27.1</v>
       </c>
       <c r="AA9">
         <v>1.18</v>
@@ -6649,7 +6649,7 @@
         <v>19.1</v>
       </c>
       <c r="AM9">
-        <v>34.3</v>
+        <v>33</v>
       </c>
       <c r="AN9">
         <v>0.006</v>
@@ -6760,7 +6760,7 @@
         <v>52.9</v>
       </c>
       <c r="BX9">
-        <v>33.1</v>
+        <v>32.3</v>
       </c>
       <c r="BY9" t="s">
         <v>208</v>
@@ -6813,7 +6813,7 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>21.2</v>
+        <v>20.5</v>
       </c>
       <c r="L10">
         <v>4</v>
@@ -6825,7 +6825,7 @@
         <v>1.98</v>
       </c>
       <c r="O10">
-        <v>23.05</v>
+        <v>20.11</v>
       </c>
       <c r="P10">
         <v>2.7</v>
@@ -6852,10 +6852,10 @@
         <v>0.1167</v>
       </c>
       <c r="X10">
-        <v>23.7</v>
+        <v>22.7</v>
       </c>
       <c r="Y10">
-        <v>88.3</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="Z10">
         <v>48.5</v>
@@ -6897,7 +6897,7 @@
         <v>89.09999999999999</v>
       </c>
       <c r="AM10">
-        <v>23.4</v>
+        <v>26.7</v>
       </c>
       <c r="AN10">
         <v>0.02</v>
@@ -7008,13 +7008,13 @@
         <v>59.1</v>
       </c>
       <c r="BX10">
-        <v>31</v>
+        <v>32.8</v>
       </c>
       <c r="BY10" t="s">
         <v>208</v>
       </c>
       <c r="BZ10">
-        <v>1.8</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="CA10" t="s">
         <v>210</v>
@@ -7058,7 +7058,7 @@
         <v>0</v>
       </c>
       <c r="K11">
-        <v>22.2</v>
+        <v>21.5</v>
       </c>
       <c r="L11">
         <v>4</v>
@@ -7070,7 +7070,7 @@
         <v>1.28</v>
       </c>
       <c r="O11">
-        <v>20.23</v>
+        <v>21.55</v>
       </c>
       <c r="P11">
         <v>6.9</v>
@@ -7097,10 +7097,10 @@
         <v>0.1167</v>
       </c>
       <c r="X11">
-        <v>22.3</v>
+        <v>22.7</v>
       </c>
       <c r="Y11">
-        <v>89</v>
+        <v>88.8</v>
       </c>
       <c r="Z11">
         <v>51.7</v>
@@ -7142,7 +7142,7 @@
         <v>81.90000000000001</v>
       </c>
       <c r="AM11">
-        <v>16.2</v>
+        <v>14.2</v>
       </c>
       <c r="AN11">
         <v>0.001</v>
@@ -7253,13 +7253,13 @@
         <v>61.3</v>
       </c>
       <c r="BX11">
-        <v>20.8</v>
+        <v>19.7</v>
       </c>
       <c r="BY11" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="BZ11">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="CA11" t="s">
         <v>210</v>
@@ -7303,7 +7303,7 @@
         <v>0</v>
       </c>
       <c r="K12">
-        <v>23.2</v>
+        <v>22.5</v>
       </c>
       <c r="L12">
         <v>4</v>
@@ -7548,7 +7548,7 @@
         <v>0</v>
       </c>
       <c r="K13">
-        <v>24.2</v>
+        <v>23.5</v>
       </c>
       <c r="L13">
         <v>4</v>
@@ -7793,10 +7793,10 @@
         <v>361</v>
       </c>
       <c r="J14">
-        <v>188.5</v>
+        <v>228.8</v>
       </c>
       <c r="K14">
-        <v>21.3</v>
+        <v>20.6</v>
       </c>
       <c r="L14">
         <v>5</v>
@@ -7997,7 +7997,7 @@
         <v>210</v>
       </c>
       <c r="BZ14">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
       <c r="CA14" t="s">
         <v>210</v>
@@ -8044,10 +8044,10 @@
         <v>361</v>
       </c>
       <c r="J15">
-        <v>188.5</v>
+        <v>228.8</v>
       </c>
       <c r="K15">
-        <v>22.3</v>
+        <v>21.6</v>
       </c>
       <c r="L15">
         <v>5</v>
@@ -8295,10 +8295,10 @@
         <v>361</v>
       </c>
       <c r="J16">
-        <v>188.5</v>
+        <v>228.8</v>
       </c>
       <c r="K16">
-        <v>23.3</v>
+        <v>22.6</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -8499,7 +8499,7 @@
         <v>210</v>
       </c>
       <c r="BZ16">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="CA16" t="s">
         <v>210</v>
@@ -8546,10 +8546,10 @@
         <v>361</v>
       </c>
       <c r="J17">
-        <v>188.5</v>
+        <v>228.8</v>
       </c>
       <c r="K17">
-        <v>24.3</v>
+        <v>23.6</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -8591,7 +8591,7 @@
         <v>11.6</v>
       </c>
       <c r="Y17">
-        <v>92.09999999999999</v>
+        <v>92.2</v>
       </c>
       <c r="Z17">
         <v>68.3</v>
@@ -8750,7 +8750,7 @@
         <v>210</v>
       </c>
       <c r="BZ17">
-        <v>4.8</v>
+        <v>4.7</v>
       </c>
       <c r="CA17" t="s">
         <v>210</v>
@@ -8797,10 +8797,10 @@
         <v>362</v>
       </c>
       <c r="J18">
-        <v>106.7</v>
+        <v>147</v>
       </c>
       <c r="K18">
-        <v>22.2</v>
+        <v>21.5</v>
       </c>
       <c r="L18">
         <v>5</v>
@@ -8812,7 +8812,7 @@
         <v>4.54</v>
       </c>
       <c r="O18">
-        <v>27.34</v>
+        <v>29.7</v>
       </c>
       <c r="P18">
         <v>7.6</v>
@@ -8839,13 +8839,13 @@
         <v>0.0833</v>
       </c>
       <c r="X18">
-        <v>47</v>
+        <v>47.8</v>
       </c>
       <c r="Y18">
-        <v>63.6</v>
+        <v>63.2</v>
       </c>
       <c r="Z18">
-        <v>74.59999999999999</v>
+        <v>74.5</v>
       </c>
       <c r="AA18">
         <v>0.98</v>
@@ -8884,7 +8884,7 @@
         <v>70.09999999999999</v>
       </c>
       <c r="AM18">
-        <v>61.3</v>
+        <v>59.8</v>
       </c>
       <c r="AN18">
         <v>0.005</v>
@@ -8962,7 +8962,7 @@
         <v>139</v>
       </c>
       <c r="BM18">
-        <v>88.59999999999999</v>
+        <v>88.7</v>
       </c>
       <c r="BN18">
         <v>8.800000000000001</v>
@@ -8989,13 +8989,13 @@
         <v>64.7</v>
       </c>
       <c r="BV18">
-        <v>59.1</v>
+        <v>59.3</v>
       </c>
       <c r="BW18">
         <v>33.7</v>
       </c>
       <c r="BX18">
-        <v>49.6</v>
+        <v>48.8</v>
       </c>
       <c r="BY18" t="s">
         <v>209</v>
@@ -9048,10 +9048,10 @@
         <v>362</v>
       </c>
       <c r="J19">
-        <v>106.7</v>
+        <v>147</v>
       </c>
       <c r="K19">
-        <v>23.2</v>
+        <v>22.5</v>
       </c>
       <c r="L19">
         <v>5</v>
@@ -9063,7 +9063,7 @@
         <v>5.92</v>
       </c>
       <c r="O19">
-        <v>20.17</v>
+        <v>25.57</v>
       </c>
       <c r="P19">
         <v>20.4</v>
@@ -9090,13 +9090,13 @@
         <v>0.0833</v>
       </c>
       <c r="X19">
-        <v>29.3</v>
+        <v>31.2</v>
       </c>
       <c r="Y19">
-        <v>71.5</v>
+        <v>70.7</v>
       </c>
       <c r="Z19">
-        <v>73.40000000000001</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="AA19">
         <v>0.98</v>
@@ -9252,7 +9252,7 @@
         <v>211</v>
       </c>
       <c r="BZ19">
-        <v>27.9</v>
+        <v>27.8</v>
       </c>
       <c r="CA19" t="s">
         <v>213</v>
@@ -9299,10 +9299,10 @@
         <v>362</v>
       </c>
       <c r="J20">
-        <v>106.7</v>
+        <v>147</v>
       </c>
       <c r="K20">
-        <v>24.2</v>
+        <v>23.5</v>
       </c>
       <c r="L20">
         <v>5</v>
@@ -9314,7 +9314,7 @@
         <v>2.61</v>
       </c>
       <c r="O20">
-        <v>23.65</v>
+        <v>18.34</v>
       </c>
       <c r="P20">
         <v>10.5</v>
@@ -9341,13 +9341,13 @@
         <v>0.0833</v>
       </c>
       <c r="X20">
-        <v>20.9</v>
+        <v>19</v>
       </c>
       <c r="Y20">
-        <v>81.5</v>
+        <v>82.3</v>
       </c>
       <c r="Z20">
-        <v>75.90000000000001</v>
+        <v>76.2</v>
       </c>
       <c r="AA20">
         <v>0.98</v>
@@ -9550,10 +9550,10 @@
         <v>362</v>
       </c>
       <c r="J21">
-        <v>106.7</v>
+        <v>147</v>
       </c>
       <c r="K21">
-        <v>25.2</v>
+        <v>24.5</v>
       </c>
       <c r="L21">
         <v>5</v>
@@ -9565,7 +9565,7 @@
         <v>3.53</v>
       </c>
       <c r="O21">
-        <v>20.13</v>
+        <v>17.64</v>
       </c>
       <c r="P21">
         <v>13.6</v>
@@ -9592,13 +9592,13 @@
         <v>0.0833</v>
       </c>
       <c r="X21">
-        <v>21.9</v>
+        <v>21</v>
       </c>
       <c r="Y21">
-        <v>75.40000000000001</v>
+        <v>75.8</v>
       </c>
       <c r="Z21">
-        <v>74.8</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="AA21">
         <v>0.98</v>
@@ -9801,10 +9801,10 @@
         <v>363</v>
       </c>
       <c r="J22">
-        <v>213.2</v>
+        <v>253.5</v>
       </c>
       <c r="K22">
-        <v>22.2</v>
+        <v>21.6</v>
       </c>
       <c r="L22">
         <v>5</v>
@@ -10005,7 +10005,7 @@
         <v>212</v>
       </c>
       <c r="BZ22">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="CA22" t="s">
         <v>210</v>
@@ -10052,10 +10052,10 @@
         <v>363</v>
       </c>
       <c r="J23">
-        <v>213.2</v>
+        <v>253.5</v>
       </c>
       <c r="K23">
-        <v>23.2</v>
+        <v>22.6</v>
       </c>
       <c r="L23">
         <v>5</v>
@@ -10256,7 +10256,7 @@
         <v>212</v>
       </c>
       <c r="BZ23">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="CA23" t="s">
         <v>210</v>
@@ -10303,10 +10303,10 @@
         <v>363</v>
       </c>
       <c r="J24">
-        <v>213.2</v>
+        <v>253.5</v>
       </c>
       <c r="K24">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L24">
         <v>5</v>
@@ -10507,7 +10507,7 @@
         <v>212</v>
       </c>
       <c r="BZ24">
-        <v>9.9</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="CA24" t="s">
         <v>210</v>
@@ -10554,10 +10554,10 @@
         <v>363</v>
       </c>
       <c r="J25">
-        <v>213.2</v>
+        <v>253.5</v>
       </c>
       <c r="K25">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -10758,7 +10758,7 @@
         <v>212</v>
       </c>
       <c r="BZ25">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="CA25" t="s">
         <v>210</v>
@@ -10805,10 +10805,10 @@
         <v>364</v>
       </c>
       <c r="J26">
-        <v>27.6</v>
+        <v>67.8</v>
       </c>
       <c r="K26">
-        <v>22.2</v>
+        <v>21.6</v>
       </c>
       <c r="L26">
         <v>5</v>
@@ -10850,7 +10850,7 @@
         <v>17</v>
       </c>
       <c r="Y26">
-        <v>87.3</v>
+        <v>87.40000000000001</v>
       </c>
       <c r="Z26">
         <v>75.40000000000001</v>
@@ -11056,10 +11056,10 @@
         <v>364</v>
       </c>
       <c r="J27">
-        <v>27.6</v>
+        <v>67.8</v>
       </c>
       <c r="K27">
-        <v>23.2</v>
+        <v>22.6</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -11260,7 +11260,7 @@
         <v>210</v>
       </c>
       <c r="BZ27">
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="CA27" t="s">
         <v>210</v>
@@ -11307,10 +11307,10 @@
         <v>364</v>
       </c>
       <c r="J28">
-        <v>27.6</v>
+        <v>67.8</v>
       </c>
       <c r="K28">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L28">
         <v>5</v>
@@ -11511,7 +11511,7 @@
         <v>210</v>
       </c>
       <c r="BZ28">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="CA28" t="s">
         <v>210</v>
@@ -11558,10 +11558,10 @@
         <v>364</v>
       </c>
       <c r="J29">
-        <v>27.6</v>
+        <v>67.8</v>
       </c>
       <c r="K29">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="L29">
         <v>5</v>
@@ -11762,7 +11762,7 @@
         <v>210</v>
       </c>
       <c r="BZ29">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="CA29" t="s">
         <v>210</v>
@@ -11809,10 +11809,10 @@
         <v>365</v>
       </c>
       <c r="J30">
-        <v>202</v>
+        <v>242.2</v>
       </c>
       <c r="K30">
-        <v>22.2</v>
+        <v>21.6</v>
       </c>
       <c r="L30">
         <v>5</v>
@@ -12060,10 +12060,10 @@
         <v>365</v>
       </c>
       <c r="J31">
-        <v>202</v>
+        <v>242.2</v>
       </c>
       <c r="K31">
-        <v>23.2</v>
+        <v>22.6</v>
       </c>
       <c r="L31">
         <v>5</v>
@@ -12311,10 +12311,10 @@
         <v>365</v>
       </c>
       <c r="J32">
-        <v>202</v>
+        <v>242.2</v>
       </c>
       <c r="K32">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -12356,7 +12356,7 @@
         <v>8.9</v>
       </c>
       <c r="Y32">
-        <v>91.8</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="Z32">
         <v>53.5</v>
@@ -12515,7 +12515,7 @@
         <v>212</v>
       </c>
       <c r="BZ32">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
       <c r="CA32" t="s">
         <v>210</v>
@@ -12562,10 +12562,10 @@
         <v>365</v>
       </c>
       <c r="J33">
-        <v>202</v>
+        <v>242.2</v>
       </c>
       <c r="K33">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="L33">
         <v>5</v>
@@ -12607,7 +12607,7 @@
         <v>12.3</v>
       </c>
       <c r="Y33">
-        <v>89.09999999999999</v>
+        <v>89.2</v>
       </c>
       <c r="Z33">
         <v>53.4</v>
@@ -12766,7 +12766,7 @@
         <v>212</v>
       </c>
       <c r="BZ33">
-        <v>9.699999999999999</v>
+        <v>9.6</v>
       </c>
       <c r="CA33" t="s">
         <v>210</v>
@@ -12813,10 +12813,10 @@
         <v>366</v>
       </c>
       <c r="J34">
-        <v>164.2</v>
+        <v>204.4</v>
       </c>
       <c r="K34">
-        <v>22.2</v>
+        <v>21.6</v>
       </c>
       <c r="L34">
         <v>5</v>
@@ -12828,7 +12828,7 @@
         <v>1.95</v>
       </c>
       <c r="O34">
-        <v>24.34</v>
+        <v>20.01</v>
       </c>
       <c r="P34">
         <v>9.699999999999999</v>
@@ -12855,13 +12855,13 @@
         <v>0.1667</v>
       </c>
       <c r="X34">
-        <v>21.5</v>
+        <v>19.9</v>
       </c>
       <c r="Y34">
-        <v>75.40000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="Z34">
-        <v>76.59999999999999</v>
+        <v>76.8</v>
       </c>
       <c r="AA34">
         <v>0.88</v>
@@ -12900,7 +12900,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="AM34">
-        <v>55.5</v>
+        <v>58.1</v>
       </c>
       <c r="AN34">
         <v>0.019</v>
@@ -12978,7 +12978,7 @@
         <v>139</v>
       </c>
       <c r="BM34">
-        <v>85.3</v>
+        <v>85.2</v>
       </c>
       <c r="BN34">
         <v>5.7</v>
@@ -12996,7 +12996,7 @@
         <v>1.085</v>
       </c>
       <c r="BS34">
-        <v>81.7</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="BT34">
         <v>85.59999999999999</v>
@@ -13005,16 +13005,16 @@
         <v>63.7</v>
       </c>
       <c r="BV34">
-        <v>56.7</v>
+        <v>56.5</v>
       </c>
       <c r="BW34">
         <v>52.7</v>
       </c>
       <c r="BX34">
-        <v>44.9</v>
+        <v>46.3</v>
       </c>
       <c r="BY34" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="BZ34">
         <v>27.1</v>
@@ -13064,10 +13064,10 @@
         <v>366</v>
       </c>
       <c r="J35">
-        <v>164.2</v>
+        <v>204.4</v>
       </c>
       <c r="K35">
-        <v>23.2</v>
+        <v>22.6</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -13079,7 +13079,7 @@
         <v>2.13</v>
       </c>
       <c r="O35">
-        <v>29.99</v>
+        <v>29.83</v>
       </c>
       <c r="P35">
         <v>8.6</v>
@@ -13106,7 +13106,7 @@
         <v>0.1667</v>
       </c>
       <c r="X35">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="Y35">
         <v>75.90000000000001</v>
@@ -13151,7 +13151,7 @@
         <v>98.5</v>
       </c>
       <c r="AM35">
-        <v>41.1</v>
+        <v>41.2</v>
       </c>
       <c r="AN35">
         <v>0.039</v>
@@ -13315,10 +13315,10 @@
         <v>366</v>
       </c>
       <c r="J36">
-        <v>164.2</v>
+        <v>204.4</v>
       </c>
       <c r="K36">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -13330,7 +13330,7 @@
         <v>1.72</v>
       </c>
       <c r="O36">
-        <v>30.63</v>
+        <v>23.39</v>
       </c>
       <c r="P36">
         <v>10.9</v>
@@ -13357,13 +13357,13 @@
         <v>0.1667</v>
       </c>
       <c r="X36">
-        <v>24.9</v>
+        <v>22.3</v>
       </c>
       <c r="Y36">
-        <v>74.90000000000001</v>
+        <v>76.09999999999999</v>
       </c>
       <c r="Z36">
-        <v>74.09999999999999</v>
+        <v>74.40000000000001</v>
       </c>
       <c r="AA36">
         <v>0.88</v>
@@ -13402,7 +13402,7 @@
         <v>98.90000000000001</v>
       </c>
       <c r="AM36">
-        <v>42</v>
+        <v>46.7</v>
       </c>
       <c r="AN36">
         <v>0.137</v>
@@ -13480,7 +13480,7 @@
         <v>139</v>
       </c>
       <c r="BM36">
-        <v>82.2</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="BN36">
         <v>5</v>
@@ -13498,7 +13498,7 @@
         <v>1.077</v>
       </c>
       <c r="BS36">
-        <v>79.2</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="BT36">
         <v>82.09999999999999</v>
@@ -13513,7 +13513,7 @@
         <v>59.8</v>
       </c>
       <c r="BX36">
-        <v>52.2</v>
+        <v>54.7</v>
       </c>
       <c r="BY36" t="s">
         <v>209</v>
@@ -13566,10 +13566,10 @@
         <v>366</v>
       </c>
       <c r="J37">
-        <v>164.2</v>
+        <v>204.4</v>
       </c>
       <c r="K37">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -13581,7 +13581,7 @@
         <v>2.43</v>
       </c>
       <c r="O37">
-        <v>27.81</v>
+        <v>24.63</v>
       </c>
       <c r="P37">
         <v>14.3</v>
@@ -13608,13 +13608,13 @@
         <v>0.1667</v>
       </c>
       <c r="X37">
-        <v>25.9</v>
+        <v>24.8</v>
       </c>
       <c r="Y37">
-        <v>71.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="Z37">
-        <v>71.40000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="AA37">
         <v>0.88</v>
@@ -13653,7 +13653,7 @@
         <v>99.59999999999999</v>
       </c>
       <c r="AM37">
-        <v>45.2</v>
+        <v>47.2</v>
       </c>
       <c r="AN37">
         <v>0.235</v>
@@ -13731,7 +13731,7 @@
         <v>139</v>
       </c>
       <c r="BM37">
-        <v>79.8</v>
+        <v>79.7</v>
       </c>
       <c r="BN37">
         <v>4.9</v>
@@ -13743,7 +13743,7 @@
         <v>1.2</v>
       </c>
       <c r="BQ37">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="BR37">
         <v>1.071</v>
@@ -13752,7 +13752,7 @@
         <v>78.40000000000001</v>
       </c>
       <c r="BT37">
-        <v>78.3</v>
+        <v>78.2</v>
       </c>
       <c r="BU37">
         <v>61.2</v>
@@ -13764,13 +13764,13 @@
         <v>66</v>
       </c>
       <c r="BX37">
-        <v>51.7</v>
+        <v>52.8</v>
       </c>
       <c r="BY37" t="s">
         <v>209</v>
       </c>
       <c r="BZ37">
-        <v>30.1</v>
+        <v>30</v>
       </c>
       <c r="CA37" t="s">
         <v>213</v>
@@ -13817,10 +13817,10 @@
         <v>367</v>
       </c>
       <c r="J38">
-        <v>208.7</v>
+        <v>248.9</v>
       </c>
       <c r="K38">
-        <v>22.2</v>
+        <v>21.6</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -13862,7 +13862,7 @@
         <v>17.8</v>
       </c>
       <c r="Y38">
-        <v>86.90000000000001</v>
+        <v>87</v>
       </c>
       <c r="Z38">
         <v>71.90000000000001</v>
@@ -14068,10 +14068,10 @@
         <v>367</v>
       </c>
       <c r="J39">
-        <v>208.7</v>
+        <v>248.9</v>
       </c>
       <c r="K39">
-        <v>23.2</v>
+        <v>22.6</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -14116,7 +14116,7 @@
         <v>85.59999999999999</v>
       </c>
       <c r="Z39">
-        <v>72.59999999999999</v>
+        <v>72.7</v>
       </c>
       <c r="AA39">
         <v>0.9399999999999999</v>
@@ -14272,7 +14272,7 @@
         <v>208</v>
       </c>
       <c r="BZ39">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="CA39" t="s">
         <v>210</v>
@@ -14319,10 +14319,10 @@
         <v>367</v>
       </c>
       <c r="J40">
-        <v>208.7</v>
+        <v>248.9</v>
       </c>
       <c r="K40">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -14364,7 +14364,7 @@
         <v>26.3</v>
       </c>
       <c r="Y40">
-        <v>83.3</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="Z40">
         <v>71.90000000000001</v>
@@ -14523,7 +14523,7 @@
         <v>208</v>
       </c>
       <c r="BZ40">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="CA40" t="s">
         <v>210</v>
@@ -14570,10 +14570,10 @@
         <v>367</v>
       </c>
       <c r="J41">
-        <v>208.7</v>
+        <v>248.9</v>
       </c>
       <c r="K41">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -14812,19 +14812,19 @@
         <v>114</v>
       </c>
       <c r="G42" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H42" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I42" t="s">
         <v>368</v>
       </c>
       <c r="J42">
-        <v>132.3</v>
+        <v>172.5</v>
       </c>
       <c r="K42">
-        <v>22.2</v>
+        <v>21.6</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -14836,7 +14836,7 @@
         <v>2.4</v>
       </c>
       <c r="O42">
-        <v>9.789999999999999</v>
+        <v>10.01</v>
       </c>
       <c r="P42">
         <v>8.699999999999999</v>
@@ -14863,7 +14863,7 @@
         <v>0.1667</v>
       </c>
       <c r="X42">
-        <v>23.6</v>
+        <v>23.7</v>
       </c>
       <c r="Y42">
         <v>86.2</v>
@@ -14908,7 +14908,7 @@
         <v>18.9</v>
       </c>
       <c r="AM42">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="AN42">
         <v>0.004</v>
@@ -15019,7 +15019,7 @@
         <v>54.6</v>
       </c>
       <c r="BX42">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="BY42" t="s">
         <v>210</v>
@@ -15063,19 +15063,19 @@
         <v>321</v>
       </c>
       <c r="G43" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H43" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I43" t="s">
         <v>368</v>
       </c>
       <c r="J43">
-        <v>132.3</v>
+        <v>172.5</v>
       </c>
       <c r="K43">
-        <v>23.2</v>
+        <v>22.6</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -15117,7 +15117,7 @@
         <v>17.1</v>
       </c>
       <c r="Y43">
-        <v>83.8</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="Z43">
         <v>54.3</v>
@@ -15276,7 +15276,7 @@
         <v>210</v>
       </c>
       <c r="BZ43">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
       <c r="CA43" t="s">
         <v>210</v>
@@ -15314,19 +15314,19 @@
         <v>322</v>
       </c>
       <c r="G44" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H44" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I44" t="s">
         <v>368</v>
       </c>
       <c r="J44">
-        <v>132.3</v>
+        <v>172.5</v>
       </c>
       <c r="K44">
-        <v>24.2</v>
+        <v>23.6</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -15565,19 +15565,19 @@
         <v>323</v>
       </c>
       <c r="G45" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H45" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="I45" t="s">
         <v>368</v>
       </c>
       <c r="J45">
-        <v>132.3</v>
+        <v>172.5</v>
       </c>
       <c r="K45">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -15589,7 +15589,7 @@
         <v>2.6</v>
       </c>
       <c r="O45">
-        <v>7.87</v>
+        <v>7.77</v>
       </c>
       <c r="P45">
         <v>12.2</v>
@@ -15616,7 +15616,7 @@
         <v>0.1667</v>
       </c>
       <c r="X45">
-        <v>12.9</v>
+        <v>12.8</v>
       </c>
       <c r="Y45">
         <v>89.09999999999999</v>
@@ -15661,7 +15661,7 @@
         <v>15.4</v>
       </c>
       <c r="AM45">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="AN45">
         <v>0.001</v>
@@ -15772,13 +15772,13 @@
         <v>63.1</v>
       </c>
       <c r="BX45">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="BY45" t="s">
         <v>210</v>
       </c>
       <c r="BZ45">
-        <v>9.4</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="CA45" t="s">
         <v>210</v>
@@ -15825,10 +15825,10 @@
         <v>359</v>
       </c>
       <c r="J46">
-        <v>112.8</v>
+        <v>153</v>
       </c>
       <c r="K46">
-        <v>25.2</v>
+        <v>24.6</v>
       </c>
       <c r="L46">
         <v>5</v>
@@ -15840,7 +15840,7 @@
         <v>1.24</v>
       </c>
       <c r="O46">
-        <v>15.14</v>
+        <v>19.53</v>
       </c>
       <c r="P46">
         <v>16.2</v>
@@ -15867,10 +15867,10 @@
         <v>0.1667</v>
       </c>
       <c r="X46">
-        <v>15</v>
+        <v>16.5</v>
       </c>
       <c r="Y46">
-        <v>84.3</v>
+        <v>83.7</v>
       </c>
       <c r="Z46">
         <v>54.8</v>
@@ -16076,10 +16076,10 @@
         <v>359</v>
       </c>
       <c r="J47">
-        <v>112.8</v>
+        <v>153</v>
       </c>
       <c r="K47">
-        <v>26.2</v>
+        <v>25.6</v>
       </c>
       <c r="L47">
         <v>5</v>
@@ -16091,7 +16091,7 @@
         <v>1.05</v>
       </c>
       <c r="O47">
-        <v>14</v>
+        <v>20.03</v>
       </c>
       <c r="P47">
         <v>24.5</v>
@@ -16118,13 +16118,13 @@
         <v>0.1667</v>
       </c>
       <c r="X47">
-        <v>12.9</v>
+        <v>15.1</v>
       </c>
       <c r="Y47">
-        <v>79.3</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="Z47">
-        <v>50.8</v>
+        <v>50.9</v>
       </c>
       <c r="AA47">
         <v>0.92</v>
@@ -16163,7 +16163,7 @@
         <v>95.5</v>
       </c>
       <c r="AM47">
-        <v>50.1</v>
+        <v>46.3</v>
       </c>
       <c r="AN47">
         <v>0.029</v>
@@ -16241,7 +16241,7 @@
         <v>139</v>
       </c>
       <c r="BM47">
-        <v>51</v>
+        <v>51.1</v>
       </c>
       <c r="BN47">
         <v>7.9</v>
@@ -16253,16 +16253,16 @@
         <v>-1.3</v>
       </c>
       <c r="BQ47">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="BR47">
-        <v>1.002</v>
+        <v>1.003</v>
       </c>
       <c r="BS47">
-        <v>55.4</v>
+        <v>55.5</v>
       </c>
       <c r="BT47">
-        <v>47.2</v>
+        <v>47.3</v>
       </c>
       <c r="BU47">
         <v>57.9</v>
@@ -16274,13 +16274,13 @@
         <v>51.3</v>
       </c>
       <c r="BX47">
-        <v>51.3</v>
+        <v>49.2</v>
       </c>
       <c r="BY47" t="s">
         <v>209</v>
       </c>
       <c r="BZ47">
-        <v>27</v>
+        <v>26.9</v>
       </c>
       <c r="CA47" t="s">
         <v>213</v>
@@ -16327,10 +16327,10 @@
         <v>359</v>
       </c>
       <c r="J48">
-        <v>112.8</v>
+        <v>153</v>
       </c>
       <c r="K48">
-        <v>27.2</v>
+        <v>26.6</v>
       </c>
       <c r="L48">
         <v>5</v>
@@ -16342,7 +16342,7 @@
         <v>1.3</v>
       </c>
       <c r="O48">
-        <v>18.68</v>
+        <v>18.6</v>
       </c>
       <c r="P48">
         <v>17.3</v>
@@ -16369,7 +16369,7 @@
         <v>0.1667</v>
       </c>
       <c r="X48">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="Y48">
         <v>80.3</v>
@@ -16525,7 +16525,7 @@
         <v>57.9</v>
       </c>
       <c r="BX48">
-        <v>58.2</v>
+        <v>58.3</v>
       </c>
       <c r="BY48" t="s">
         <v>209</v>
@@ -16578,10 +16578,10 @@
         <v>359</v>
       </c>
       <c r="J49">
-        <v>112.8</v>
+        <v>153</v>
       </c>
       <c r="K49">
-        <v>28.2</v>
+        <v>27.6</v>
       </c>
       <c r="L49">
         <v>5</v>
@@ -16593,7 +16593,7 @@
         <v>3.58</v>
       </c>
       <c r="O49">
-        <v>23.94</v>
+        <v>19.24</v>
       </c>
       <c r="P49">
         <v>8.699999999999999</v>
@@ -16620,13 +16620,13 @@
         <v>0.1667</v>
       </c>
       <c r="X49">
-        <v>21.8</v>
+        <v>20.2</v>
       </c>
       <c r="Y49">
-        <v>76.90000000000001</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="Z49">
-        <v>34.1</v>
+        <v>33.9</v>
       </c>
       <c r="AA49">
         <v>0.92</v>
@@ -16665,7 +16665,7 @@
         <v>82.5</v>
       </c>
       <c r="AM49">
-        <v>38.4</v>
+        <v>41.7</v>
       </c>
       <c r="AN49">
         <v>0.014</v>
@@ -16776,7 +16776,7 @@
         <v>59.6</v>
       </c>
       <c r="BX49">
-        <v>34</v>
+        <v>35.8</v>
       </c>
       <c r="BY49" t="s">
         <v>208</v>
@@ -16829,10 +16829,10 @@
         <v>369</v>
       </c>
       <c r="J50">
-        <v>208.3</v>
+        <v>248.5</v>
       </c>
       <c r="K50">
-        <v>26.2</v>
+        <v>25.5</v>
       </c>
       <c r="L50">
         <v>5</v>
@@ -17033,7 +17033,7 @@
         <v>210</v>
       </c>
       <c r="BZ50">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
       <c r="CA50" t="s">
         <v>210</v>
@@ -17080,10 +17080,10 @@
         <v>369</v>
       </c>
       <c r="J51">
-        <v>208.3</v>
+        <v>248.5</v>
       </c>
       <c r="K51">
-        <v>27.2</v>
+        <v>26.5</v>
       </c>
       <c r="L51">
         <v>5</v>
@@ -17284,7 +17284,7 @@
         <v>210</v>
       </c>
       <c r="BZ51">
-        <v>11.1</v>
+        <v>11</v>
       </c>
       <c r="CA51" t="s">
         <v>210</v>
@@ -17331,10 +17331,10 @@
         <v>369</v>
       </c>
       <c r="J52">
-        <v>208.3</v>
+        <v>248.5</v>
       </c>
       <c r="K52">
-        <v>28.2</v>
+        <v>27.5</v>
       </c>
       <c r="L52">
         <v>5</v>
@@ -17376,7 +17376,7 @@
         <v>8.9</v>
       </c>
       <c r="Y52">
-        <v>89.7</v>
+        <v>89.8</v>
       </c>
       <c r="Z52">
         <v>46.4</v>
@@ -17535,7 +17535,7 @@
         <v>210</v>
       </c>
       <c r="BZ52">
-        <v>11.4</v>
+        <v>11.3</v>
       </c>
       <c r="CA52" t="s">
         <v>210</v>
@@ -17582,10 +17582,10 @@
         <v>369</v>
       </c>
       <c r="J53">
-        <v>208.3</v>
+        <v>248.5</v>
       </c>
       <c r="K53">
-        <v>29.2</v>
+        <v>28.5</v>
       </c>
       <c r="L53">
         <v>5</v>
@@ -17833,10 +17833,10 @@
         <v>370</v>
       </c>
       <c r="J54">
-        <v>160.8</v>
+        <v>201</v>
       </c>
       <c r="K54">
-        <v>26.2</v>
+        <v>25.5</v>
       </c>
       <c r="L54">
         <v>5</v>
@@ -17848,7 +17848,7 @@
         <v>0.91</v>
       </c>
       <c r="O54">
-        <v>19.48</v>
+        <v>13.53</v>
       </c>
       <c r="P54">
         <v>39.9</v>
@@ -17875,13 +17875,13 @@
         <v>0.1333</v>
       </c>
       <c r="X54">
-        <v>12.1</v>
+        <v>10</v>
       </c>
       <c r="Y54">
-        <v>85.8</v>
+        <v>86.7</v>
       </c>
       <c r="Z54">
-        <v>69.5</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="AA54">
         <v>0.92</v>
@@ -17920,7 +17920,7 @@
         <v>98.5</v>
       </c>
       <c r="AM54">
-        <v>61.2</v>
+        <v>65.7</v>
       </c>
       <c r="AN54">
         <v>0.025</v>
@@ -17998,7 +17998,7 @@
         <v>139</v>
       </c>
       <c r="BM54">
-        <v>72.7</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="BN54">
         <v>6.2</v>
@@ -18010,34 +18010,34 @@
         <v>1.7</v>
       </c>
       <c r="BQ54">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="BR54">
-        <v>1.055</v>
+        <v>1.054</v>
       </c>
       <c r="BS54">
-        <v>69.2</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="BT54">
-        <v>74.7</v>
+        <v>74.59999999999999</v>
       </c>
       <c r="BU54">
         <v>61.3</v>
       </c>
       <c r="BV54">
-        <v>54.4</v>
+        <v>54</v>
       </c>
       <c r="BW54">
         <v>52</v>
       </c>
       <c r="BX54">
-        <v>55.5</v>
+        <v>58</v>
       </c>
       <c r="BY54" t="s">
         <v>209</v>
       </c>
       <c r="BZ54">
-        <v>16</v>
+        <v>15.9</v>
       </c>
       <c r="CA54" t="s">
         <v>210</v>
@@ -18084,10 +18084,10 @@
         <v>370</v>
       </c>
       <c r="J55">
-        <v>160.8</v>
+        <v>201</v>
       </c>
       <c r="K55">
-        <v>27.2</v>
+        <v>26.5</v>
       </c>
       <c r="L55">
         <v>5</v>
@@ -18099,7 +18099,7 @@
         <v>1.42</v>
       </c>
       <c r="O55">
-        <v>19.71</v>
+        <v>20.03</v>
       </c>
       <c r="P55">
         <v>26</v>
@@ -18126,7 +18126,7 @@
         <v>0.1333</v>
       </c>
       <c r="X55">
-        <v>13.9</v>
+        <v>14</v>
       </c>
       <c r="Y55">
         <v>84.8</v>
@@ -18171,7 +18171,7 @@
         <v>93.7</v>
       </c>
       <c r="AM55">
-        <v>60.9</v>
+        <v>60.5</v>
       </c>
       <c r="AN55">
         <v>0.008</v>
@@ -18264,31 +18264,31 @@
         <v>0.4</v>
       </c>
       <c r="BR55">
-        <v>1.051</v>
+        <v>1.052</v>
       </c>
       <c r="BS55">
         <v>68.90000000000001</v>
       </c>
       <c r="BT55">
-        <v>72.5</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="BU55">
         <v>60</v>
       </c>
       <c r="BV55">
-        <v>54.2</v>
+        <v>54.3</v>
       </c>
       <c r="BW55">
         <v>56.7</v>
       </c>
       <c r="BX55">
-        <v>48.7</v>
+        <v>48.5</v>
       </c>
       <c r="BY55" t="s">
         <v>209</v>
       </c>
       <c r="BZ55">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="CA55" t="s">
         <v>210</v>
@@ -18335,10 +18335,10 @@
         <v>370</v>
       </c>
       <c r="J56">
-        <v>160.8</v>
+        <v>201</v>
       </c>
       <c r="K56">
-        <v>28.2</v>
+        <v>27.5</v>
       </c>
       <c r="L56">
         <v>5</v>
@@ -18350,7 +18350,7 @@
         <v>1.47</v>
       </c>
       <c r="O56">
-        <v>25.29</v>
+        <v>24.48</v>
       </c>
       <c r="P56">
         <v>18.5</v>
@@ -18377,10 +18377,10 @@
         <v>0.1333</v>
       </c>
       <c r="X56">
-        <v>16.6</v>
+        <v>16.4</v>
       </c>
       <c r="Y56">
-        <v>83.7</v>
+        <v>83.8</v>
       </c>
       <c r="Z56">
         <v>67.40000000000001</v>
@@ -18422,7 +18422,7 @@
         <v>61.3</v>
       </c>
       <c r="AM56">
-        <v>56.8</v>
+        <v>58.3</v>
       </c>
       <c r="AN56">
         <v>0.011</v>
@@ -18521,25 +18521,25 @@
         <v>68.5</v>
       </c>
       <c r="BT56">
-        <v>71.7</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="BU56">
         <v>59.5</v>
       </c>
       <c r="BV56">
-        <v>54.5</v>
+        <v>54.4</v>
       </c>
       <c r="BW56">
         <v>58.7</v>
       </c>
       <c r="BX56">
-        <v>47.8</v>
+        <v>48.6</v>
       </c>
       <c r="BY56" t="s">
         <v>209</v>
       </c>
       <c r="BZ56">
-        <v>16.1</v>
+        <v>16</v>
       </c>
       <c r="CA56" t="s">
         <v>210</v>
@@ -18586,10 +18586,10 @@
         <v>370</v>
       </c>
       <c r="J57">
-        <v>160.8</v>
+        <v>201</v>
       </c>
       <c r="K57">
-        <v>29.2</v>
+        <v>28.5</v>
       </c>
       <c r="L57">
         <v>5</v>
@@ -18601,7 +18601,7 @@
         <v>1.81</v>
       </c>
       <c r="O57">
-        <v>26.44</v>
+        <v>24.51</v>
       </c>
       <c r="P57">
         <v>4.2</v>
@@ -18628,10 +18628,10 @@
         <v>0.1333</v>
       </c>
       <c r="X57">
-        <v>19.5</v>
+        <v>18.8</v>
       </c>
       <c r="Y57">
-        <v>77.40000000000001</v>
+        <v>77.7</v>
       </c>
       <c r="Z57">
         <v>66.90000000000001</v>
@@ -18673,7 +18673,7 @@
         <v>97.40000000000001</v>
       </c>
       <c r="AM57">
-        <v>51</v>
+        <v>53.9</v>
       </c>
       <c r="AN57">
         <v>0.023</v>
@@ -18763,16 +18763,16 @@
         <v>0</v>
       </c>
       <c r="BQ57">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="BR57">
         <v>1.052</v>
       </c>
       <c r="BS57">
-        <v>69.90000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="BT57">
-        <v>72.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="BU57">
         <v>59.5</v>
@@ -18784,7 +18784,7 @@
         <v>60.8</v>
       </c>
       <c r="BX57">
-        <v>49.2</v>
+        <v>50.8</v>
       </c>
       <c r="BY57" t="s">
         <v>209</v>
@@ -18837,10 +18837,10 @@
         <v>371</v>
       </c>
       <c r="J58">
-        <v>54.1</v>
+        <v>94.3</v>
       </c>
       <c r="K58">
-        <v>28.2</v>
+        <v>27.5</v>
       </c>
       <c r="L58">
         <v>5</v>
@@ -18882,7 +18882,7 @@
         <v>8.699999999999999</v>
       </c>
       <c r="Y58">
-        <v>88.8</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="Z58">
         <v>75.7</v>
@@ -19088,10 +19088,10 @@
         <v>371</v>
       </c>
       <c r="J59">
-        <v>54.1</v>
+        <v>94.3</v>
       </c>
       <c r="K59">
-        <v>29.2</v>
+        <v>28.5</v>
       </c>
       <c r="L59">
         <v>5</v>
@@ -19339,10 +19339,10 @@
         <v>371</v>
       </c>
       <c r="J60">
-        <v>54.1</v>
+        <v>94.3</v>
       </c>
       <c r="K60">
-        <v>30.2</v>
+        <v>29.5</v>
       </c>
       <c r="L60">
         <v>5</v>
@@ -19543,7 +19543,7 @@
         <v>210</v>
       </c>
       <c r="BZ60">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="CA60" t="s">
         <v>210</v>
@@ -19590,10 +19590,10 @@
         <v>371</v>
       </c>
       <c r="J61">
-        <v>54.1</v>
+        <v>94.3</v>
       </c>
       <c r="K61">
-        <v>31.2</v>
+        <v>30.5</v>
       </c>
       <c r="L61">
         <v>5</v>
@@ -19841,10 +19841,10 @@
         <v>372</v>
       </c>
       <c r="J62">
-        <v>6.4</v>
+        <v>46.6</v>
       </c>
       <c r="K62">
-        <v>28.2</v>
+        <v>27.5</v>
       </c>
       <c r="L62">
         <v>5</v>
@@ -20045,7 +20045,7 @@
         <v>210</v>
       </c>
       <c r="BZ62">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
       <c r="CA62" t="s">
         <v>210</v>
@@ -20092,10 +20092,10 @@
         <v>372</v>
       </c>
       <c r="J63">
-        <v>6.4</v>
+        <v>46.6</v>
       </c>
       <c r="K63">
-        <v>29.2</v>
+        <v>28.5</v>
       </c>
       <c r="L63">
         <v>5</v>
@@ -20296,7 +20296,7 @@
         <v>210</v>
       </c>
       <c r="BZ63">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="CA63" t="s">
         <v>210</v>
@@ -20343,10 +20343,10 @@
         <v>372</v>
       </c>
       <c r="J64">
-        <v>6.4</v>
+        <v>46.6</v>
       </c>
       <c r="K64">
-        <v>30.2</v>
+        <v>29.5</v>
       </c>
       <c r="L64">
         <v>5</v>
@@ -20547,7 +20547,7 @@
         <v>210</v>
       </c>
       <c r="BZ64">
-        <v>8.5</v>
+        <v>8.4</v>
       </c>
       <c r="CA64" t="s">
         <v>210</v>
@@ -20594,10 +20594,10 @@
         <v>372</v>
       </c>
       <c r="J65">
-        <v>6.4</v>
+        <v>46.6</v>
       </c>
       <c r="K65">
-        <v>31.2</v>
+        <v>30.5</v>
       </c>
       <c r="L65">
         <v>5</v>
@@ -20798,7 +20798,7 @@
         <v>210</v>
       </c>
       <c r="BZ65">
-        <v>10.3</v>
+        <v>10.2</v>
       </c>
       <c r="CA65" t="s">
         <v>210</v>
@@ -20974,7 +20974,7 @@
         <v>181</v>
       </c>
       <c r="G3">
-        <v>70.7</v>
+        <v>70.5</v>
       </c>
       <c r="H3">
         <v>11</v>
@@ -21027,7 +21027,7 @@
         <v>181</v>
       </c>
       <c r="G4">
-        <v>85.2</v>
+        <v>85.3</v>
       </c>
       <c r="H4">
         <v>11</v>
@@ -21074,13 +21074,13 @@
         <v>130</v>
       </c>
       <c r="E5">
-        <v>65.2</v>
+        <v>65.3</v>
       </c>
       <c r="F5" t="s">
         <v>181</v>
       </c>
       <c r="G5">
-        <v>75.09999999999999</v>
+        <v>75.7</v>
       </c>
       <c r="H5">
         <v>9</v>
@@ -21133,7 +21133,7 @@
         <v>181</v>
       </c>
       <c r="G6">
-        <v>89.7</v>
+        <v>89.8</v>
       </c>
       <c r="H6">
         <v>9</v>
@@ -21239,7 +21239,7 @@
         <v>181</v>
       </c>
       <c r="G8">
-        <v>84.2</v>
+        <v>84.7</v>
       </c>
       <c r="H8">
         <v>8</v>
@@ -21292,7 +21292,7 @@
         <v>181</v>
       </c>
       <c r="G9">
-        <v>75</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="H9">
         <v>8</v>
@@ -21504,7 +21504,7 @@
         <v>182</v>
       </c>
       <c r="G13">
-        <v>81.3</v>
+        <v>80.8</v>
       </c>
       <c r="H13">
         <v>3</v>
@@ -21557,7 +21557,7 @@
         <v>182</v>
       </c>
       <c r="G14">
-        <v>88.8</v>
+        <v>87.2</v>
       </c>
       <c r="H14">
         <v>2</v>
@@ -21663,7 +21663,7 @@
         <v>182</v>
       </c>
       <c r="G16">
-        <v>88.3</v>
+        <v>88.40000000000001</v>
       </c>
       <c r="H16">
         <v>0</v>

</xml_diff>